<commit_message>
Add Preconditions column to test cases, remove repeated first steps
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/saucedemo-test-cases/Demo_test_cases.xlsx
+++ b/saucedemo-test-cases/Demo_test_cases.xlsx
@@ -598,13 +598,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -620,10 +621,15 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Expected result</t>
         </is>
@@ -642,13 +648,17 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>1. Open the login page
-2. Enter username standard_user
-3. Enter password secret_sauce
-4. Click Login</t>
+          <t>Login page is open</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>1. Enter username standard_user
+2. Enter password secret_sauce
+3. Click Login</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>User lands on the Products page.</t>
         </is>
@@ -667,13 +677,17 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>1. Open the login page
-2. Enter username standard_user
-3. Enter password wrong
-4. Click Login</t>
+          <t>Login page is open</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>1. Enter username standard_user
+2. Enter password wrong
+3. Click Login</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Error "Username and password do not match any user in this service" is shown. User stays on the login page.</t>
         </is>
@@ -692,13 +706,17 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>1. Open the login page
-2. Leave username empty
-3. Enter password secret_sauce
-4. Click Login</t>
+          <t>Login page is open</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>1. Leave username empty
+2. Enter password secret_sauce
+3. Click Login</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Error "Username is required" is shown.</t>
         </is>
@@ -717,13 +735,17 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>1. Open the login page
-2. Enter username standard_user
-3. Leave password empty
-4. Click Login</t>
+          <t>Login page is open</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>1. Enter username standard_user
+2. Leave password empty
+3. Click Login</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Error "Password is required" is shown.</t>
         </is>
@@ -742,13 +764,17 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>1. Open the login page
-2. Enter username locked_out_user
-3. Enter password secret_sauce
-4. Click Login</t>
+          <t>Login page is open</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>1. Enter username locked_out_user
+2. Enter password secret_sauce
+3. Click Login</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Error "Sorry, this user has been locked out" is shown.</t>
         </is>
@@ -767,11 +793,15 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>1. Open a new browser session
-2. Open /inventory.html directly</t>
+          <t>New browser session, user is not logged in</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>1. Open /inventory.html directly</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Access is denied and an error is shown on the login page.</t>
         </is>
@@ -790,13 +820,17 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>1. Log in as standard_user
-2. Open the menu
-3. Click Logout
-4. Click the browser Back button</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>1. Open the menu
+2. Click Logout
+3. Click the browser Back button</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>User returns to the login page. Back button does not reopen the Products page as logged in.</t>
         </is>
@@ -815,13 +849,17 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>1. Open the login page
-2. Enter username STANDARD_USER
-3. Enter password secret_sauce
-4. Click Login</t>
+          <t>Login page is open</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>1. Enter username STANDARD_USER
+2. Enter password secret_sauce
+3. Click Login</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Login is rejected.</t>
         </is>
@@ -840,11 +878,16 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>1. Trigger any login error
+          <t>Login page is open</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>1. Click Login with empty fields to trigger an error
 2. Click the X on the error message</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>The message disappears.</t>
         </is>
@@ -861,13 +904,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -883,10 +927,15 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Expected result</t>
         </is>
@@ -905,10 +954,15 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>1. Log in as standard_user</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>1. Open the Products page</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>6 products are shown, each with image, name, description, price and Add to cart button.</t>
         </is>
@@ -927,11 +981,15 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Select "Name (A to Z)" in the sort dropdown</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>1. Select "Name (A to Z)" in the sort dropdown</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Products are sorted alphabetically, ascending.</t>
         </is>
@@ -950,11 +1008,15 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Select "Name (Z to A)" in the sort dropdown</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>1. Select "Name (Z to A)" in the sort dropdown</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Products are sorted alphabetically, descending.</t>
         </is>
@@ -973,11 +1035,15 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Select "Price (low to high)" in the sort dropdown</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>1. Select "Price (low to high)" in the sort dropdown</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Prices are in ascending order.</t>
         </is>
@@ -996,11 +1062,15 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Select "Price (high to low)" in the sort dropdown</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>1. Select "Price (high to low)" in the sort dropdown</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Prices are in descending order.</t>
         </is>
@@ -1019,11 +1089,15 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Click a product name</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>1. Click a product name</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Details page shows the same name, description and price as the catalog.</t>
         </is>
@@ -1042,11 +1116,15 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>1. Open a product details page
-2. Click "Back to products"</t>
+          <t>Product details page is open</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>1. Click "Back to products"</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>The catalog is shown.</t>
         </is>
@@ -1065,11 +1143,15 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Compare every product image with its name</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>1. Compare every product image with its name</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Each image corresponds to its product.</t>
         </is>
@@ -1086,13 +1168,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1108,10 +1191,15 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Expected result</t>
         </is>
@@ -1130,11 +1218,15 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Click "Add to cart" on one product</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>1. Click "Add to cart" on one product</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Button changes to "Remove". Cart badge shows 1.</t>
         </is>
@@ -1153,12 +1245,16 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Add 3 different products
-3. Open the cart</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>1. Add 3 different products
+2. Open the cart</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Badge shows 3. Cart page lists the 3 products.</t>
         </is>
@@ -1177,12 +1273,16 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Add a product
-3. Click "Remove" on the same product</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>1. Add a product
+2. Click "Remove" on the same product</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Badge disappears or decreases. Button returns to "Add to cart".</t>
         </is>
@@ -1201,13 +1301,17 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Add a product
-3. Open the cart
-4. Click Remove</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>1. Add a product
+2. Open the cart
+3. Click Remove</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Item is removed from the list. Badge updates.</t>
         </is>
@@ -1226,13 +1330,17 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Add a product
-3. Open its details page
-4. Click "Back to products"</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>1. Add a product
+2. Open its details page
+3. Click "Back to products"</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Item is still in the cart and the button still says "Remove".</t>
         </is>
@@ -1251,13 +1359,17 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Add a product
-3. Log out
-4. Log in again</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>1. Add a product
+2. Log out
+3. Log in again</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Observed behavior is recorded and compared with the expectation (cart saved or cleared).</t>
         </is>
@@ -1276,12 +1388,16 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>1. Add a product
-2. Open the cart
-3. Click "Continue Shopping"</t>
+          <t>User is logged in, cart has a product</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>1. Open the cart
+2. Click "Continue Shopping"</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Catalog is shown and the cart is unchanged.</t>
         </is>
@@ -1300,12 +1416,16 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Open the empty cart
-3. Click Checkout</t>
+          <t>User is logged in as standard_user, cart is empty</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>1. Open the cart
+2. Click Checkout</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Observed behavior is recorded. A purchase with zero items should not be possible.</t>
         </is>
@@ -1322,13 +1442,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1344,10 +1465,15 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Expected result</t>
         </is>
@@ -1366,15 +1492,19 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>1. Log in
-2. Add a product
-3. Open the cart and click Checkout
-4. Enter first name, last name and postal code
-5. Click Continue
-6. Click Finish</t>
+          <t>User is logged in as standard_user</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>1. Add a product
+2. Open the cart and click Checkout
+3. Enter first name, last name and postal code
+4. Click Continue
+5. Click Finish</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Overview shows correct items and totals. Confirmation "Thank you for your order" is shown. Cart is empty.</t>
         </is>
@@ -1393,12 +1523,16 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>1. Go to checkout step one
-2. Leave first name empty, fill other fields
-3. Click Continue</t>
+          <t>Checkout step one page is open (cart has a product)</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>1. Leave first name empty, fill other fields
+2. Click Continue</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Error "First Name is required" is shown.</t>
         </is>
@@ -1417,12 +1551,16 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>1. Go to checkout step one
-2. Leave last name empty, fill other fields
-3. Click Continue</t>
+          <t>Checkout step one page is open (cart has a product)</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>1. Leave last name empty, fill other fields
+2. Click Continue</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Error "Last Name is required" is shown.</t>
         </is>
@@ -1441,12 +1579,16 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>1. Go to checkout step one
-2. Leave postal code empty, fill other fields
-3. Click Continue</t>
+          <t>Checkout step one page is open (cart has a product)</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>1. Leave postal code empty, fill other fields
+2. Click Continue</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Error "Postal Code is required" is shown.</t>
         </is>
@@ -1465,11 +1607,16 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
+          <t>User is logged in as standard_user</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
           <t>1. Add 2 products with known prices
 2. Go through checkout to the overview page</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Item total equals the sum of prices. Total equals item total plus tax.</t>
         </is>
@@ -1488,11 +1635,16 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
+          <t>User is logged in as standard_user</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
           <t>1. Add 2 products
 2. Go through checkout to the overview page</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>The same products and quantities as in the cart are listed.</t>
         </is>
@@ -1511,11 +1663,15 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>1. Go to checkout step one
-2. Click Cancel</t>
+          <t>Checkout step one page is open (cart has a product)</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>1. Click Cancel</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>User returns to the cart and items are preserved.</t>
         </is>
@@ -1534,11 +1690,15 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>1. Go to the overview page
-2. Click Cancel</t>
+          <t>Checkout overview page is open (cart has a product)</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>1. Click Cancel</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>User returns to the catalog and items are preserved.</t>
         </is>
@@ -1557,13 +1717,17 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>1. Go to checkout step one
-2. Enter &lt;script&gt;alert(1)&lt;/script&gt; as first name
-3. Fill other fields
-4. Click Continue</t>
+          <t>Checkout step one page is open (cart has a product)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>1. Enter &lt;script&gt;alert(1)&lt;/script&gt; as first name
+2. Fill other fields
+3. Click Continue</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Input is handled as plain text and no script runs.</t>
         </is>
@@ -1582,12 +1746,16 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>1. Go to checkout step one
-2. Enter 300 characters in each field
-3. Click Continue</t>
+          <t>Checkout step one page is open (cart has a product)</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>1. Enter 300 characters in each field
+2. Click Continue</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>No crash and no broken layout. Observed behavior is recorded.</t>
         </is>
@@ -1606,11 +1774,15 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>1. Complete a checkout
-2. Click "Back Home"</t>
+          <t>Order is completed (confirmation page is shown)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>1. Click "Back Home"</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Catalog is shown and the cart is empty.</t>
         </is>
@@ -1627,13 +1799,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1649,10 +1822,15 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Expected result</t>
         </is>
@@ -1671,10 +1849,15 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
+          <t>Chrome, Firefox and Edge are installed</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
           <t>1. Run the scenarios above in each browser</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>All scenarios behave the same.</t>
         </is>
@@ -1693,11 +1876,16 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
+          <t>User is logged in as standard_user</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
           <t>1. Resize the browser window to 375 px width
-2. Go through login, catalog, cart and checkout</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
+2. Go through catalog, cart and checkout</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Layout is usable. Nothing overlaps or is cut off.</t>
         </is>
@@ -1716,11 +1904,16 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
+          <t>Login page is open</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
           <t>1. Use only Tab and Enter
-2. Complete the login and checkout forms</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
+2. Log in and complete the checkout forms</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Forms can be completed without a mouse.</t>
         </is>

</xml_diff>